<commit_message>
Review queue, inline rename and colour/size switches on Products.
Products gets ALL / IN REVIEW / LIVE / DRAFT tabs, click-to-rename, and
PUBLISH / UNPUBLISH per row (with the reason when publishing is refused).
Each row expands into its colours (image + on/off switch) and each colour's
sizes (on/off chips). New products start in review; the product sheet
template drops its Status column since publishing now happens here.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/SunoBro-Product-Sheet.xlsx
+++ b/public/SunoBro-Product-Sheet.xlsx
@@ -552,7 +552,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>One row per product (e.g. 'Unisex Classic Crew T-Shirt'). Name, description, selling price, status and cover image.</t>
+          <t>One row per product. Give every design its own name (e.g. 'Eventual Consistency Tee'), not Qikink's generic 'Unisex Classic Crew T-Shirt'. Name, description, selling price, cover image.</t>
         </is>
       </c>
     </row>
@@ -607,12 +607,12 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Going live</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>active = visible on the site (only if every variant has a Store SKU — see 'Ready to publish'). draft = saved but hidden.</t>
+          <t>The sheet never publishes. New products arrive in admin → Products → IN REVIEW; check them and click PUBLISH. You can also switch individual colours or sizes off there.</t>
         </is>
       </c>
     </row>
@@ -624,7 +624,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Re-upload the same sheet after edits. Products are matched by Product name; variants by colour + size. Remove a row to remove that variant.</t>
+          <t>Re-upload the same sheet after edits. Products are matched by URL slug, then Product name; variants by colour + size. Remove a row to remove that variant. Live/draft status and switched-off colours are kept.</t>
         </is>
       </c>
     </row>
@@ -715,22 +715,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M60"/>
+  <dimension ref="A1:L60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="44" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -751,50 +750,45 @@
       </c>
       <c r="D1" s="8" t="inlineStr">
         <is>
-          <t>Status *</t>
-        </is>
-      </c>
-      <c r="E1" s="8" t="inlineStr">
-        <is>
           <t>Cover image URL *</t>
         </is>
       </c>
-      <c r="F1" s="8" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>More image URLs (separate with |)</t>
         </is>
       </c>
-      <c r="G1" s="8" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>URL slug (auto if blank)</t>
         </is>
       </c>
-      <c r="H1" s="8" t="inlineStr">
+      <c r="G1" s="8" t="inlineStr">
         <is>
           <t>Qikink Product ID</t>
         </is>
       </c>
-      <c r="I1" s="8" t="inlineStr">
+      <c r="H1" s="8" t="inlineStr">
         <is>
           <t>Design name</t>
         </is>
       </c>
-      <c r="J1" s="8" t="inlineStr">
+      <c r="I1" s="8" t="inlineStr">
         <is>
           <t>Print size (W × H in)</t>
         </is>
       </c>
-      <c r="K1" s="8" t="inlineStr">
+      <c r="J1" s="8" t="inlineStr">
         <is>
           <t>Variants</t>
         </is>
       </c>
-      <c r="L1" s="8" t="inlineStr">
+      <c r="K1" s="8" t="inlineStr">
         <is>
           <t>With Store SKU</t>
         </is>
       </c>
-      <c r="M1" s="8" t="inlineStr">
+      <c r="L1" s="8" t="inlineStr">
         <is>
           <t>Ready to publish</t>
         </is>
@@ -816,45 +810,40 @@
       </c>
       <c r="D2" s="9" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="E2" s="9" t="inlineStr">
-        <is>
           <t>https://qikink-assets.s3.ap-south-1.amazonaws.com/clients/621544/clientProducts/32422268/images/Front_1_c_1.jpg</t>
         </is>
       </c>
-      <c r="F2" s="11" t="n"/>
-      <c r="G2" s="11" t="inlineStr">
+      <c r="E2" s="11" t="n"/>
+      <c r="F2" s="11" t="inlineStr">
         <is>
           <t>unisex-classic-crew-t-shirt</t>
         </is>
       </c>
-      <c r="H2" s="11" t="inlineStr">
+      <c r="G2" s="11" t="inlineStr">
         <is>
           <t>64844536</t>
         </is>
       </c>
-      <c r="I2" s="11" t="inlineStr">
+      <c r="H2" s="11" t="inlineStr">
         <is>
           <t>imgtext</t>
         </is>
       </c>
-      <c r="J2" s="11" t="inlineStr">
+      <c r="I2" s="11" t="inlineStr">
         <is>
           <t>14 × 6.4</t>
         </is>
       </c>
+      <c r="J2" s="12">
+        <f>IF(A2="","",COUNTIF(Variants!$A:$A,A2))</f>
+        <v/>
+      </c>
       <c r="K2" s="12">
-        <f>IF(A2="","",COUNTIF(Variants!$A:$A,A2))</f>
+        <f>IF(A2="","",COUNTIFS(Variants!$A:$A,A2,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L2" s="12">
-        <f>IF(A2="","",COUNTIFS(Variants!$A:$A,A2,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M2" s="12">
-        <f>IF(A2="","",IF(K2=0,"ADD VARIANTS",IF(L2&lt;K2,"MISSING "&amp;(K2-L2)&amp;" STORE SKU",IF(E2="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A2="","",IF(J2=0,"ADD VARIANTS",IF(K2&lt;J2,"MISSING "&amp;(J2-K2)&amp;" STORE SKU",IF(D2="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -863,22 +852,21 @@
       <c r="B3" s="9" t="n"/>
       <c r="C3" s="10" t="n"/>
       <c r="D3" s="9" t="n"/>
-      <c r="E3" s="9" t="n"/>
+      <c r="E3" s="11" t="n"/>
       <c r="F3" s="11" t="n"/>
       <c r="G3" s="11" t="n"/>
       <c r="H3" s="11" t="n"/>
       <c r="I3" s="11" t="n"/>
-      <c r="J3" s="11" t="n"/>
+      <c r="J3" s="12">
+        <f>IF(A3="","",COUNTIF(Variants!$A:$A,A3))</f>
+        <v/>
+      </c>
       <c r="K3" s="12">
-        <f>IF(A3="","",COUNTIF(Variants!$A:$A,A3))</f>
+        <f>IF(A3="","",COUNTIFS(Variants!$A:$A,A3,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L3" s="12">
-        <f>IF(A3="","",COUNTIFS(Variants!$A:$A,A3,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M3" s="12">
-        <f>IF(A3="","",IF(K3=0,"ADD VARIANTS",IF(L3&lt;K3,"MISSING "&amp;(K3-L3)&amp;" STORE SKU",IF(E3="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A3="","",IF(J3=0,"ADD VARIANTS",IF(K3&lt;J3,"MISSING "&amp;(J3-K3)&amp;" STORE SKU",IF(D3="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -887,22 +875,21 @@
       <c r="B4" s="9" t="n"/>
       <c r="C4" s="10" t="n"/>
       <c r="D4" s="9" t="n"/>
-      <c r="E4" s="9" t="n"/>
+      <c r="E4" s="11" t="n"/>
       <c r="F4" s="11" t="n"/>
       <c r="G4" s="11" t="n"/>
       <c r="H4" s="11" t="n"/>
       <c r="I4" s="11" t="n"/>
-      <c r="J4" s="11" t="n"/>
+      <c r="J4" s="12">
+        <f>IF(A4="","",COUNTIF(Variants!$A:$A,A4))</f>
+        <v/>
+      </c>
       <c r="K4" s="12">
-        <f>IF(A4="","",COUNTIF(Variants!$A:$A,A4))</f>
+        <f>IF(A4="","",COUNTIFS(Variants!$A:$A,A4,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L4" s="12">
-        <f>IF(A4="","",COUNTIFS(Variants!$A:$A,A4,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M4" s="12">
-        <f>IF(A4="","",IF(K4=0,"ADD VARIANTS",IF(L4&lt;K4,"MISSING "&amp;(K4-L4)&amp;" STORE SKU",IF(E4="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A4="","",IF(J4=0,"ADD VARIANTS",IF(K4&lt;J4,"MISSING "&amp;(J4-K4)&amp;" STORE SKU",IF(D4="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -911,22 +898,21 @@
       <c r="B5" s="9" t="n"/>
       <c r="C5" s="10" t="n"/>
       <c r="D5" s="9" t="n"/>
-      <c r="E5" s="9" t="n"/>
+      <c r="E5" s="11" t="n"/>
       <c r="F5" s="11" t="n"/>
       <c r="G5" s="11" t="n"/>
       <c r="H5" s="11" t="n"/>
       <c r="I5" s="11" t="n"/>
-      <c r="J5" s="11" t="n"/>
+      <c r="J5" s="12">
+        <f>IF(A5="","",COUNTIF(Variants!$A:$A,A5))</f>
+        <v/>
+      </c>
       <c r="K5" s="12">
-        <f>IF(A5="","",COUNTIF(Variants!$A:$A,A5))</f>
+        <f>IF(A5="","",COUNTIFS(Variants!$A:$A,A5,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L5" s="12">
-        <f>IF(A5="","",COUNTIFS(Variants!$A:$A,A5,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M5" s="12">
-        <f>IF(A5="","",IF(K5=0,"ADD VARIANTS",IF(L5&lt;K5,"MISSING "&amp;(K5-L5)&amp;" STORE SKU",IF(E5="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A5="","",IF(J5=0,"ADD VARIANTS",IF(K5&lt;J5,"MISSING "&amp;(J5-K5)&amp;" STORE SKU",IF(D5="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -935,22 +921,21 @@
       <c r="B6" s="9" t="n"/>
       <c r="C6" s="10" t="n"/>
       <c r="D6" s="9" t="n"/>
-      <c r="E6" s="9" t="n"/>
+      <c r="E6" s="11" t="n"/>
       <c r="F6" s="11" t="n"/>
       <c r="G6" s="11" t="n"/>
       <c r="H6" s="11" t="n"/>
       <c r="I6" s="11" t="n"/>
-      <c r="J6" s="11" t="n"/>
+      <c r="J6" s="12">
+        <f>IF(A6="","",COUNTIF(Variants!$A:$A,A6))</f>
+        <v/>
+      </c>
       <c r="K6" s="12">
-        <f>IF(A6="","",COUNTIF(Variants!$A:$A,A6))</f>
+        <f>IF(A6="","",COUNTIFS(Variants!$A:$A,A6,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L6" s="12">
-        <f>IF(A6="","",COUNTIFS(Variants!$A:$A,A6,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M6" s="12">
-        <f>IF(A6="","",IF(K6=0,"ADD VARIANTS",IF(L6&lt;K6,"MISSING "&amp;(K6-L6)&amp;" STORE SKU",IF(E6="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A6="","",IF(J6=0,"ADD VARIANTS",IF(K6&lt;J6,"MISSING "&amp;(J6-K6)&amp;" STORE SKU",IF(D6="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -959,22 +944,21 @@
       <c r="B7" s="9" t="n"/>
       <c r="C7" s="10" t="n"/>
       <c r="D7" s="9" t="n"/>
-      <c r="E7" s="9" t="n"/>
+      <c r="E7" s="11" t="n"/>
       <c r="F7" s="11" t="n"/>
       <c r="G7" s="11" t="n"/>
       <c r="H7" s="11" t="n"/>
       <c r="I7" s="11" t="n"/>
-      <c r="J7" s="11" t="n"/>
+      <c r="J7" s="12">
+        <f>IF(A7="","",COUNTIF(Variants!$A:$A,A7))</f>
+        <v/>
+      </c>
       <c r="K7" s="12">
-        <f>IF(A7="","",COUNTIF(Variants!$A:$A,A7))</f>
+        <f>IF(A7="","",COUNTIFS(Variants!$A:$A,A7,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L7" s="12">
-        <f>IF(A7="","",COUNTIFS(Variants!$A:$A,A7,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M7" s="12">
-        <f>IF(A7="","",IF(K7=0,"ADD VARIANTS",IF(L7&lt;K7,"MISSING "&amp;(K7-L7)&amp;" STORE SKU",IF(E7="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A7="","",IF(J7=0,"ADD VARIANTS",IF(K7&lt;J7,"MISSING "&amp;(J7-K7)&amp;" STORE SKU",IF(D7="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -983,22 +967,21 @@
       <c r="B8" s="9" t="n"/>
       <c r="C8" s="10" t="n"/>
       <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
+      <c r="E8" s="11" t="n"/>
       <c r="F8" s="11" t="n"/>
       <c r="G8" s="11" t="n"/>
       <c r="H8" s="11" t="n"/>
       <c r="I8" s="11" t="n"/>
-      <c r="J8" s="11" t="n"/>
+      <c r="J8" s="12">
+        <f>IF(A8="","",COUNTIF(Variants!$A:$A,A8))</f>
+        <v/>
+      </c>
       <c r="K8" s="12">
-        <f>IF(A8="","",COUNTIF(Variants!$A:$A,A8))</f>
+        <f>IF(A8="","",COUNTIFS(Variants!$A:$A,A8,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L8" s="12">
-        <f>IF(A8="","",COUNTIFS(Variants!$A:$A,A8,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M8" s="12">
-        <f>IF(A8="","",IF(K8=0,"ADD VARIANTS",IF(L8&lt;K8,"MISSING "&amp;(K8-L8)&amp;" STORE SKU",IF(E8="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A8="","",IF(J8=0,"ADD VARIANTS",IF(K8&lt;J8,"MISSING "&amp;(J8-K8)&amp;" STORE SKU",IF(D8="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1007,22 +990,21 @@
       <c r="B9" s="9" t="n"/>
       <c r="C9" s="10" t="n"/>
       <c r="D9" s="9" t="n"/>
-      <c r="E9" s="9" t="n"/>
+      <c r="E9" s="11" t="n"/>
       <c r="F9" s="11" t="n"/>
       <c r="G9" s="11" t="n"/>
       <c r="H9" s="11" t="n"/>
       <c r="I9" s="11" t="n"/>
-      <c r="J9" s="11" t="n"/>
+      <c r="J9" s="12">
+        <f>IF(A9="","",COUNTIF(Variants!$A:$A,A9))</f>
+        <v/>
+      </c>
       <c r="K9" s="12">
-        <f>IF(A9="","",COUNTIF(Variants!$A:$A,A9))</f>
+        <f>IF(A9="","",COUNTIFS(Variants!$A:$A,A9,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L9" s="12">
-        <f>IF(A9="","",COUNTIFS(Variants!$A:$A,A9,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M9" s="12">
-        <f>IF(A9="","",IF(K9=0,"ADD VARIANTS",IF(L9&lt;K9,"MISSING "&amp;(K9-L9)&amp;" STORE SKU",IF(E9="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A9="","",IF(J9=0,"ADD VARIANTS",IF(K9&lt;J9,"MISSING "&amp;(J9-K9)&amp;" STORE SKU",IF(D9="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1031,22 +1013,21 @@
       <c r="B10" s="9" t="n"/>
       <c r="C10" s="10" t="n"/>
       <c r="D10" s="9" t="n"/>
-      <c r="E10" s="9" t="n"/>
+      <c r="E10" s="11" t="n"/>
       <c r="F10" s="11" t="n"/>
       <c r="G10" s="11" t="n"/>
       <c r="H10" s="11" t="n"/>
       <c r="I10" s="11" t="n"/>
-      <c r="J10" s="11" t="n"/>
+      <c r="J10" s="12">
+        <f>IF(A10="","",COUNTIF(Variants!$A:$A,A10))</f>
+        <v/>
+      </c>
       <c r="K10" s="12">
-        <f>IF(A10="","",COUNTIF(Variants!$A:$A,A10))</f>
+        <f>IF(A10="","",COUNTIFS(Variants!$A:$A,A10,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L10" s="12">
-        <f>IF(A10="","",COUNTIFS(Variants!$A:$A,A10,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M10" s="12">
-        <f>IF(A10="","",IF(K10=0,"ADD VARIANTS",IF(L10&lt;K10,"MISSING "&amp;(K10-L10)&amp;" STORE SKU",IF(E10="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A10="","",IF(J10=0,"ADD VARIANTS",IF(K10&lt;J10,"MISSING "&amp;(J10-K10)&amp;" STORE SKU",IF(D10="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1055,22 +1036,21 @@
       <c r="B11" s="9" t="n"/>
       <c r="C11" s="10" t="n"/>
       <c r="D11" s="9" t="n"/>
-      <c r="E11" s="9" t="n"/>
+      <c r="E11" s="11" t="n"/>
       <c r="F11" s="11" t="n"/>
       <c r="G11" s="11" t="n"/>
       <c r="H11" s="11" t="n"/>
       <c r="I11" s="11" t="n"/>
-      <c r="J11" s="11" t="n"/>
+      <c r="J11" s="12">
+        <f>IF(A11="","",COUNTIF(Variants!$A:$A,A11))</f>
+        <v/>
+      </c>
       <c r="K11" s="12">
-        <f>IF(A11="","",COUNTIF(Variants!$A:$A,A11))</f>
+        <f>IF(A11="","",COUNTIFS(Variants!$A:$A,A11,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L11" s="12">
-        <f>IF(A11="","",COUNTIFS(Variants!$A:$A,A11,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M11" s="12">
-        <f>IF(A11="","",IF(K11=0,"ADD VARIANTS",IF(L11&lt;K11,"MISSING "&amp;(K11-L11)&amp;" STORE SKU",IF(E11="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A11="","",IF(J11=0,"ADD VARIANTS",IF(K11&lt;J11,"MISSING "&amp;(J11-K11)&amp;" STORE SKU",IF(D11="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1079,22 +1059,21 @@
       <c r="B12" s="9" t="n"/>
       <c r="C12" s="10" t="n"/>
       <c r="D12" s="9" t="n"/>
-      <c r="E12" s="9" t="n"/>
+      <c r="E12" s="11" t="n"/>
       <c r="F12" s="11" t="n"/>
       <c r="G12" s="11" t="n"/>
       <c r="H12" s="11" t="n"/>
       <c r="I12" s="11" t="n"/>
-      <c r="J12" s="11" t="n"/>
+      <c r="J12" s="12">
+        <f>IF(A12="","",COUNTIF(Variants!$A:$A,A12))</f>
+        <v/>
+      </c>
       <c r="K12" s="12">
-        <f>IF(A12="","",COUNTIF(Variants!$A:$A,A12))</f>
+        <f>IF(A12="","",COUNTIFS(Variants!$A:$A,A12,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L12" s="12">
-        <f>IF(A12="","",COUNTIFS(Variants!$A:$A,A12,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M12" s="12">
-        <f>IF(A12="","",IF(K12=0,"ADD VARIANTS",IF(L12&lt;K12,"MISSING "&amp;(K12-L12)&amp;" STORE SKU",IF(E12="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A12="","",IF(J12=0,"ADD VARIANTS",IF(K12&lt;J12,"MISSING "&amp;(J12-K12)&amp;" STORE SKU",IF(D12="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1103,22 +1082,21 @@
       <c r="B13" s="9" t="n"/>
       <c r="C13" s="10" t="n"/>
       <c r="D13" s="9" t="n"/>
-      <c r="E13" s="9" t="n"/>
+      <c r="E13" s="11" t="n"/>
       <c r="F13" s="11" t="n"/>
       <c r="G13" s="11" t="n"/>
       <c r="H13" s="11" t="n"/>
       <c r="I13" s="11" t="n"/>
-      <c r="J13" s="11" t="n"/>
+      <c r="J13" s="12">
+        <f>IF(A13="","",COUNTIF(Variants!$A:$A,A13))</f>
+        <v/>
+      </c>
       <c r="K13" s="12">
-        <f>IF(A13="","",COUNTIF(Variants!$A:$A,A13))</f>
+        <f>IF(A13="","",COUNTIFS(Variants!$A:$A,A13,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L13" s="12">
-        <f>IF(A13="","",COUNTIFS(Variants!$A:$A,A13,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M13" s="12">
-        <f>IF(A13="","",IF(K13=0,"ADD VARIANTS",IF(L13&lt;K13,"MISSING "&amp;(K13-L13)&amp;" STORE SKU",IF(E13="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A13="","",IF(J13=0,"ADD VARIANTS",IF(K13&lt;J13,"MISSING "&amp;(J13-K13)&amp;" STORE SKU",IF(D13="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1127,22 +1105,21 @@
       <c r="B14" s="9" t="n"/>
       <c r="C14" s="10" t="n"/>
       <c r="D14" s="9" t="n"/>
-      <c r="E14" s="9" t="n"/>
+      <c r="E14" s="11" t="n"/>
       <c r="F14" s="11" t="n"/>
       <c r="G14" s="11" t="n"/>
       <c r="H14" s="11" t="n"/>
       <c r="I14" s="11" t="n"/>
-      <c r="J14" s="11" t="n"/>
+      <c r="J14" s="12">
+        <f>IF(A14="","",COUNTIF(Variants!$A:$A,A14))</f>
+        <v/>
+      </c>
       <c r="K14" s="12">
-        <f>IF(A14="","",COUNTIF(Variants!$A:$A,A14))</f>
+        <f>IF(A14="","",COUNTIFS(Variants!$A:$A,A14,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L14" s="12">
-        <f>IF(A14="","",COUNTIFS(Variants!$A:$A,A14,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M14" s="12">
-        <f>IF(A14="","",IF(K14=0,"ADD VARIANTS",IF(L14&lt;K14,"MISSING "&amp;(K14-L14)&amp;" STORE SKU",IF(E14="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A14="","",IF(J14=0,"ADD VARIANTS",IF(K14&lt;J14,"MISSING "&amp;(J14-K14)&amp;" STORE SKU",IF(D14="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1151,22 +1128,21 @@
       <c r="B15" s="9" t="n"/>
       <c r="C15" s="10" t="n"/>
       <c r="D15" s="9" t="n"/>
-      <c r="E15" s="9" t="n"/>
+      <c r="E15" s="11" t="n"/>
       <c r="F15" s="11" t="n"/>
       <c r="G15" s="11" t="n"/>
       <c r="H15" s="11" t="n"/>
       <c r="I15" s="11" t="n"/>
-      <c r="J15" s="11" t="n"/>
+      <c r="J15" s="12">
+        <f>IF(A15="","",COUNTIF(Variants!$A:$A,A15))</f>
+        <v/>
+      </c>
       <c r="K15" s="12">
-        <f>IF(A15="","",COUNTIF(Variants!$A:$A,A15))</f>
+        <f>IF(A15="","",COUNTIFS(Variants!$A:$A,A15,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L15" s="12">
-        <f>IF(A15="","",COUNTIFS(Variants!$A:$A,A15,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M15" s="12">
-        <f>IF(A15="","",IF(K15=0,"ADD VARIANTS",IF(L15&lt;K15,"MISSING "&amp;(K15-L15)&amp;" STORE SKU",IF(E15="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A15="","",IF(J15=0,"ADD VARIANTS",IF(K15&lt;J15,"MISSING "&amp;(J15-K15)&amp;" STORE SKU",IF(D15="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1175,22 +1151,21 @@
       <c r="B16" s="9" t="n"/>
       <c r="C16" s="10" t="n"/>
       <c r="D16" s="9" t="n"/>
-      <c r="E16" s="9" t="n"/>
+      <c r="E16" s="11" t="n"/>
       <c r="F16" s="11" t="n"/>
       <c r="G16" s="11" t="n"/>
       <c r="H16" s="11" t="n"/>
       <c r="I16" s="11" t="n"/>
-      <c r="J16" s="11" t="n"/>
+      <c r="J16" s="12">
+        <f>IF(A16="","",COUNTIF(Variants!$A:$A,A16))</f>
+        <v/>
+      </c>
       <c r="K16" s="12">
-        <f>IF(A16="","",COUNTIF(Variants!$A:$A,A16))</f>
+        <f>IF(A16="","",COUNTIFS(Variants!$A:$A,A16,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L16" s="12">
-        <f>IF(A16="","",COUNTIFS(Variants!$A:$A,A16,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M16" s="12">
-        <f>IF(A16="","",IF(K16=0,"ADD VARIANTS",IF(L16&lt;K16,"MISSING "&amp;(K16-L16)&amp;" STORE SKU",IF(E16="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A16="","",IF(J16=0,"ADD VARIANTS",IF(K16&lt;J16,"MISSING "&amp;(J16-K16)&amp;" STORE SKU",IF(D16="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1199,22 +1174,21 @@
       <c r="B17" s="9" t="n"/>
       <c r="C17" s="10" t="n"/>
       <c r="D17" s="9" t="n"/>
-      <c r="E17" s="9" t="n"/>
+      <c r="E17" s="11" t="n"/>
       <c r="F17" s="11" t="n"/>
       <c r="G17" s="11" t="n"/>
       <c r="H17" s="11" t="n"/>
       <c r="I17" s="11" t="n"/>
-      <c r="J17" s="11" t="n"/>
+      <c r="J17" s="12">
+        <f>IF(A17="","",COUNTIF(Variants!$A:$A,A17))</f>
+        <v/>
+      </c>
       <c r="K17" s="12">
-        <f>IF(A17="","",COUNTIF(Variants!$A:$A,A17))</f>
+        <f>IF(A17="","",COUNTIFS(Variants!$A:$A,A17,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L17" s="12">
-        <f>IF(A17="","",COUNTIFS(Variants!$A:$A,A17,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M17" s="12">
-        <f>IF(A17="","",IF(K17=0,"ADD VARIANTS",IF(L17&lt;K17,"MISSING "&amp;(K17-L17)&amp;" STORE SKU",IF(E17="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A17="","",IF(J17=0,"ADD VARIANTS",IF(K17&lt;J17,"MISSING "&amp;(J17-K17)&amp;" STORE SKU",IF(D17="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1223,22 +1197,21 @@
       <c r="B18" s="9" t="n"/>
       <c r="C18" s="10" t="n"/>
       <c r="D18" s="9" t="n"/>
-      <c r="E18" s="9" t="n"/>
+      <c r="E18" s="11" t="n"/>
       <c r="F18" s="11" t="n"/>
       <c r="G18" s="11" t="n"/>
       <c r="H18" s="11" t="n"/>
       <c r="I18" s="11" t="n"/>
-      <c r="J18" s="11" t="n"/>
+      <c r="J18" s="12">
+        <f>IF(A18="","",COUNTIF(Variants!$A:$A,A18))</f>
+        <v/>
+      </c>
       <c r="K18" s="12">
-        <f>IF(A18="","",COUNTIF(Variants!$A:$A,A18))</f>
+        <f>IF(A18="","",COUNTIFS(Variants!$A:$A,A18,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L18" s="12">
-        <f>IF(A18="","",COUNTIFS(Variants!$A:$A,A18,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M18" s="12">
-        <f>IF(A18="","",IF(K18=0,"ADD VARIANTS",IF(L18&lt;K18,"MISSING "&amp;(K18-L18)&amp;" STORE SKU",IF(E18="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A18="","",IF(J18=0,"ADD VARIANTS",IF(K18&lt;J18,"MISSING "&amp;(J18-K18)&amp;" STORE SKU",IF(D18="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1247,22 +1220,21 @@
       <c r="B19" s="9" t="n"/>
       <c r="C19" s="10" t="n"/>
       <c r="D19" s="9" t="n"/>
-      <c r="E19" s="9" t="n"/>
+      <c r="E19" s="11" t="n"/>
       <c r="F19" s="11" t="n"/>
       <c r="G19" s="11" t="n"/>
       <c r="H19" s="11" t="n"/>
       <c r="I19" s="11" t="n"/>
-      <c r="J19" s="11" t="n"/>
+      <c r="J19" s="12">
+        <f>IF(A19="","",COUNTIF(Variants!$A:$A,A19))</f>
+        <v/>
+      </c>
       <c r="K19" s="12">
-        <f>IF(A19="","",COUNTIF(Variants!$A:$A,A19))</f>
+        <f>IF(A19="","",COUNTIFS(Variants!$A:$A,A19,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L19" s="12">
-        <f>IF(A19="","",COUNTIFS(Variants!$A:$A,A19,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M19" s="12">
-        <f>IF(A19="","",IF(K19=0,"ADD VARIANTS",IF(L19&lt;K19,"MISSING "&amp;(K19-L19)&amp;" STORE SKU",IF(E19="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A19="","",IF(J19=0,"ADD VARIANTS",IF(K19&lt;J19,"MISSING "&amp;(J19-K19)&amp;" STORE SKU",IF(D19="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1271,22 +1243,21 @@
       <c r="B20" s="9" t="n"/>
       <c r="C20" s="10" t="n"/>
       <c r="D20" s="9" t="n"/>
-      <c r="E20" s="9" t="n"/>
+      <c r="E20" s="11" t="n"/>
       <c r="F20" s="11" t="n"/>
       <c r="G20" s="11" t="n"/>
       <c r="H20" s="11" t="n"/>
       <c r="I20" s="11" t="n"/>
-      <c r="J20" s="11" t="n"/>
+      <c r="J20" s="12">
+        <f>IF(A20="","",COUNTIF(Variants!$A:$A,A20))</f>
+        <v/>
+      </c>
       <c r="K20" s="12">
-        <f>IF(A20="","",COUNTIF(Variants!$A:$A,A20))</f>
+        <f>IF(A20="","",COUNTIFS(Variants!$A:$A,A20,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L20" s="12">
-        <f>IF(A20="","",COUNTIFS(Variants!$A:$A,A20,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M20" s="12">
-        <f>IF(A20="","",IF(K20=0,"ADD VARIANTS",IF(L20&lt;K20,"MISSING "&amp;(K20-L20)&amp;" STORE SKU",IF(E20="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A20="","",IF(J20=0,"ADD VARIANTS",IF(K20&lt;J20,"MISSING "&amp;(J20-K20)&amp;" STORE SKU",IF(D20="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1295,22 +1266,21 @@
       <c r="B21" s="9" t="n"/>
       <c r="C21" s="10" t="n"/>
       <c r="D21" s="9" t="n"/>
-      <c r="E21" s="9" t="n"/>
+      <c r="E21" s="11" t="n"/>
       <c r="F21" s="11" t="n"/>
       <c r="G21" s="11" t="n"/>
       <c r="H21" s="11" t="n"/>
       <c r="I21" s="11" t="n"/>
-      <c r="J21" s="11" t="n"/>
+      <c r="J21" s="12">
+        <f>IF(A21="","",COUNTIF(Variants!$A:$A,A21))</f>
+        <v/>
+      </c>
       <c r="K21" s="12">
-        <f>IF(A21="","",COUNTIF(Variants!$A:$A,A21))</f>
+        <f>IF(A21="","",COUNTIFS(Variants!$A:$A,A21,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L21" s="12">
-        <f>IF(A21="","",COUNTIFS(Variants!$A:$A,A21,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M21" s="12">
-        <f>IF(A21="","",IF(K21=0,"ADD VARIANTS",IF(L21&lt;K21,"MISSING "&amp;(K21-L21)&amp;" STORE SKU",IF(E21="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A21="","",IF(J21=0,"ADD VARIANTS",IF(K21&lt;J21,"MISSING "&amp;(J21-K21)&amp;" STORE SKU",IF(D21="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1319,22 +1289,21 @@
       <c r="B22" s="9" t="n"/>
       <c r="C22" s="10" t="n"/>
       <c r="D22" s="9" t="n"/>
-      <c r="E22" s="9" t="n"/>
+      <c r="E22" s="11" t="n"/>
       <c r="F22" s="11" t="n"/>
       <c r="G22" s="11" t="n"/>
       <c r="H22" s="11" t="n"/>
       <c r="I22" s="11" t="n"/>
-      <c r="J22" s="11" t="n"/>
+      <c r="J22" s="12">
+        <f>IF(A22="","",COUNTIF(Variants!$A:$A,A22))</f>
+        <v/>
+      </c>
       <c r="K22" s="12">
-        <f>IF(A22="","",COUNTIF(Variants!$A:$A,A22))</f>
+        <f>IF(A22="","",COUNTIFS(Variants!$A:$A,A22,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L22" s="12">
-        <f>IF(A22="","",COUNTIFS(Variants!$A:$A,A22,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M22" s="12">
-        <f>IF(A22="","",IF(K22=0,"ADD VARIANTS",IF(L22&lt;K22,"MISSING "&amp;(K22-L22)&amp;" STORE SKU",IF(E22="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A22="","",IF(J22=0,"ADD VARIANTS",IF(K22&lt;J22,"MISSING "&amp;(J22-K22)&amp;" STORE SKU",IF(D22="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1343,22 +1312,21 @@
       <c r="B23" s="9" t="n"/>
       <c r="C23" s="10" t="n"/>
       <c r="D23" s="9" t="n"/>
-      <c r="E23" s="9" t="n"/>
+      <c r="E23" s="11" t="n"/>
       <c r="F23" s="11" t="n"/>
       <c r="G23" s="11" t="n"/>
       <c r="H23" s="11" t="n"/>
       <c r="I23" s="11" t="n"/>
-      <c r="J23" s="11" t="n"/>
+      <c r="J23" s="12">
+        <f>IF(A23="","",COUNTIF(Variants!$A:$A,A23))</f>
+        <v/>
+      </c>
       <c r="K23" s="12">
-        <f>IF(A23="","",COUNTIF(Variants!$A:$A,A23))</f>
+        <f>IF(A23="","",COUNTIFS(Variants!$A:$A,A23,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L23" s="12">
-        <f>IF(A23="","",COUNTIFS(Variants!$A:$A,A23,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M23" s="12">
-        <f>IF(A23="","",IF(K23=0,"ADD VARIANTS",IF(L23&lt;K23,"MISSING "&amp;(K23-L23)&amp;" STORE SKU",IF(E23="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A23="","",IF(J23=0,"ADD VARIANTS",IF(K23&lt;J23,"MISSING "&amp;(J23-K23)&amp;" STORE SKU",IF(D23="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1367,22 +1335,21 @@
       <c r="B24" s="9" t="n"/>
       <c r="C24" s="10" t="n"/>
       <c r="D24" s="9" t="n"/>
-      <c r="E24" s="9" t="n"/>
+      <c r="E24" s="11" t="n"/>
       <c r="F24" s="11" t="n"/>
       <c r="G24" s="11" t="n"/>
       <c r="H24" s="11" t="n"/>
       <c r="I24" s="11" t="n"/>
-      <c r="J24" s="11" t="n"/>
+      <c r="J24" s="12">
+        <f>IF(A24="","",COUNTIF(Variants!$A:$A,A24))</f>
+        <v/>
+      </c>
       <c r="K24" s="12">
-        <f>IF(A24="","",COUNTIF(Variants!$A:$A,A24))</f>
+        <f>IF(A24="","",COUNTIFS(Variants!$A:$A,A24,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L24" s="12">
-        <f>IF(A24="","",COUNTIFS(Variants!$A:$A,A24,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M24" s="12">
-        <f>IF(A24="","",IF(K24=0,"ADD VARIANTS",IF(L24&lt;K24,"MISSING "&amp;(K24-L24)&amp;" STORE SKU",IF(E24="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A24="","",IF(J24=0,"ADD VARIANTS",IF(K24&lt;J24,"MISSING "&amp;(J24-K24)&amp;" STORE SKU",IF(D24="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1391,22 +1358,21 @@
       <c r="B25" s="9" t="n"/>
       <c r="C25" s="10" t="n"/>
       <c r="D25" s="9" t="n"/>
-      <c r="E25" s="9" t="n"/>
+      <c r="E25" s="11" t="n"/>
       <c r="F25" s="11" t="n"/>
       <c r="G25" s="11" t="n"/>
       <c r="H25" s="11" t="n"/>
       <c r="I25" s="11" t="n"/>
-      <c r="J25" s="11" t="n"/>
+      <c r="J25" s="12">
+        <f>IF(A25="","",COUNTIF(Variants!$A:$A,A25))</f>
+        <v/>
+      </c>
       <c r="K25" s="12">
-        <f>IF(A25="","",COUNTIF(Variants!$A:$A,A25))</f>
+        <f>IF(A25="","",COUNTIFS(Variants!$A:$A,A25,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L25" s="12">
-        <f>IF(A25="","",COUNTIFS(Variants!$A:$A,A25,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M25" s="12">
-        <f>IF(A25="","",IF(K25=0,"ADD VARIANTS",IF(L25&lt;K25,"MISSING "&amp;(K25-L25)&amp;" STORE SKU",IF(E25="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A25="","",IF(J25=0,"ADD VARIANTS",IF(K25&lt;J25,"MISSING "&amp;(J25-K25)&amp;" STORE SKU",IF(D25="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1415,22 +1381,21 @@
       <c r="B26" s="9" t="n"/>
       <c r="C26" s="10" t="n"/>
       <c r="D26" s="9" t="n"/>
-      <c r="E26" s="9" t="n"/>
+      <c r="E26" s="11" t="n"/>
       <c r="F26" s="11" t="n"/>
       <c r="G26" s="11" t="n"/>
       <c r="H26" s="11" t="n"/>
       <c r="I26" s="11" t="n"/>
-      <c r="J26" s="11" t="n"/>
+      <c r="J26" s="12">
+        <f>IF(A26="","",COUNTIF(Variants!$A:$A,A26))</f>
+        <v/>
+      </c>
       <c r="K26" s="12">
-        <f>IF(A26="","",COUNTIF(Variants!$A:$A,A26))</f>
+        <f>IF(A26="","",COUNTIFS(Variants!$A:$A,A26,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L26" s="12">
-        <f>IF(A26="","",COUNTIFS(Variants!$A:$A,A26,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M26" s="12">
-        <f>IF(A26="","",IF(K26=0,"ADD VARIANTS",IF(L26&lt;K26,"MISSING "&amp;(K26-L26)&amp;" STORE SKU",IF(E26="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A26="","",IF(J26=0,"ADD VARIANTS",IF(K26&lt;J26,"MISSING "&amp;(J26-K26)&amp;" STORE SKU",IF(D26="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1439,22 +1404,21 @@
       <c r="B27" s="9" t="n"/>
       <c r="C27" s="10" t="n"/>
       <c r="D27" s="9" t="n"/>
-      <c r="E27" s="9" t="n"/>
+      <c r="E27" s="11" t="n"/>
       <c r="F27" s="11" t="n"/>
       <c r="G27" s="11" t="n"/>
       <c r="H27" s="11" t="n"/>
       <c r="I27" s="11" t="n"/>
-      <c r="J27" s="11" t="n"/>
+      <c r="J27" s="12">
+        <f>IF(A27="","",COUNTIF(Variants!$A:$A,A27))</f>
+        <v/>
+      </c>
       <c r="K27" s="12">
-        <f>IF(A27="","",COUNTIF(Variants!$A:$A,A27))</f>
+        <f>IF(A27="","",COUNTIFS(Variants!$A:$A,A27,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L27" s="12">
-        <f>IF(A27="","",COUNTIFS(Variants!$A:$A,A27,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M27" s="12">
-        <f>IF(A27="","",IF(K27=0,"ADD VARIANTS",IF(L27&lt;K27,"MISSING "&amp;(K27-L27)&amp;" STORE SKU",IF(E27="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A27="","",IF(J27=0,"ADD VARIANTS",IF(K27&lt;J27,"MISSING "&amp;(J27-K27)&amp;" STORE SKU",IF(D27="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1463,22 +1427,21 @@
       <c r="B28" s="9" t="n"/>
       <c r="C28" s="10" t="n"/>
       <c r="D28" s="9" t="n"/>
-      <c r="E28" s="9" t="n"/>
+      <c r="E28" s="11" t="n"/>
       <c r="F28" s="11" t="n"/>
       <c r="G28" s="11" t="n"/>
       <c r="H28" s="11" t="n"/>
       <c r="I28" s="11" t="n"/>
-      <c r="J28" s="11" t="n"/>
+      <c r="J28" s="12">
+        <f>IF(A28="","",COUNTIF(Variants!$A:$A,A28))</f>
+        <v/>
+      </c>
       <c r="K28" s="12">
-        <f>IF(A28="","",COUNTIF(Variants!$A:$A,A28))</f>
+        <f>IF(A28="","",COUNTIFS(Variants!$A:$A,A28,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L28" s="12">
-        <f>IF(A28="","",COUNTIFS(Variants!$A:$A,A28,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M28" s="12">
-        <f>IF(A28="","",IF(K28=0,"ADD VARIANTS",IF(L28&lt;K28,"MISSING "&amp;(K28-L28)&amp;" STORE SKU",IF(E28="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A28="","",IF(J28=0,"ADD VARIANTS",IF(K28&lt;J28,"MISSING "&amp;(J28-K28)&amp;" STORE SKU",IF(D28="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1487,22 +1450,21 @@
       <c r="B29" s="9" t="n"/>
       <c r="C29" s="10" t="n"/>
       <c r="D29" s="9" t="n"/>
-      <c r="E29" s="9" t="n"/>
+      <c r="E29" s="11" t="n"/>
       <c r="F29" s="11" t="n"/>
       <c r="G29" s="11" t="n"/>
       <c r="H29" s="11" t="n"/>
       <c r="I29" s="11" t="n"/>
-      <c r="J29" s="11" t="n"/>
+      <c r="J29" s="12">
+        <f>IF(A29="","",COUNTIF(Variants!$A:$A,A29))</f>
+        <v/>
+      </c>
       <c r="K29" s="12">
-        <f>IF(A29="","",COUNTIF(Variants!$A:$A,A29))</f>
+        <f>IF(A29="","",COUNTIFS(Variants!$A:$A,A29,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L29" s="12">
-        <f>IF(A29="","",COUNTIFS(Variants!$A:$A,A29,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M29" s="12">
-        <f>IF(A29="","",IF(K29=0,"ADD VARIANTS",IF(L29&lt;K29,"MISSING "&amp;(K29-L29)&amp;" STORE SKU",IF(E29="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A29="","",IF(J29=0,"ADD VARIANTS",IF(K29&lt;J29,"MISSING "&amp;(J29-K29)&amp;" STORE SKU",IF(D29="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1511,22 +1473,21 @@
       <c r="B30" s="9" t="n"/>
       <c r="C30" s="10" t="n"/>
       <c r="D30" s="9" t="n"/>
-      <c r="E30" s="9" t="n"/>
+      <c r="E30" s="11" t="n"/>
       <c r="F30" s="11" t="n"/>
       <c r="G30" s="11" t="n"/>
       <c r="H30" s="11" t="n"/>
       <c r="I30" s="11" t="n"/>
-      <c r="J30" s="11" t="n"/>
+      <c r="J30" s="12">
+        <f>IF(A30="","",COUNTIF(Variants!$A:$A,A30))</f>
+        <v/>
+      </c>
       <c r="K30" s="12">
-        <f>IF(A30="","",COUNTIF(Variants!$A:$A,A30))</f>
+        <f>IF(A30="","",COUNTIFS(Variants!$A:$A,A30,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L30" s="12">
-        <f>IF(A30="","",COUNTIFS(Variants!$A:$A,A30,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M30" s="12">
-        <f>IF(A30="","",IF(K30=0,"ADD VARIANTS",IF(L30&lt;K30,"MISSING "&amp;(K30-L30)&amp;" STORE SKU",IF(E30="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A30="","",IF(J30=0,"ADD VARIANTS",IF(K30&lt;J30,"MISSING "&amp;(J30-K30)&amp;" STORE SKU",IF(D30="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1535,22 +1496,21 @@
       <c r="B31" s="9" t="n"/>
       <c r="C31" s="10" t="n"/>
       <c r="D31" s="9" t="n"/>
-      <c r="E31" s="9" t="n"/>
+      <c r="E31" s="11" t="n"/>
       <c r="F31" s="11" t="n"/>
       <c r="G31" s="11" t="n"/>
       <c r="H31" s="11" t="n"/>
       <c r="I31" s="11" t="n"/>
-      <c r="J31" s="11" t="n"/>
+      <c r="J31" s="12">
+        <f>IF(A31="","",COUNTIF(Variants!$A:$A,A31))</f>
+        <v/>
+      </c>
       <c r="K31" s="12">
-        <f>IF(A31="","",COUNTIF(Variants!$A:$A,A31))</f>
+        <f>IF(A31="","",COUNTIFS(Variants!$A:$A,A31,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L31" s="12">
-        <f>IF(A31="","",COUNTIFS(Variants!$A:$A,A31,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M31" s="12">
-        <f>IF(A31="","",IF(K31=0,"ADD VARIANTS",IF(L31&lt;K31,"MISSING "&amp;(K31-L31)&amp;" STORE SKU",IF(E31="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A31="","",IF(J31=0,"ADD VARIANTS",IF(K31&lt;J31,"MISSING "&amp;(J31-K31)&amp;" STORE SKU",IF(D31="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1559,22 +1519,21 @@
       <c r="B32" s="9" t="n"/>
       <c r="C32" s="10" t="n"/>
       <c r="D32" s="9" t="n"/>
-      <c r="E32" s="9" t="n"/>
+      <c r="E32" s="11" t="n"/>
       <c r="F32" s="11" t="n"/>
       <c r="G32" s="11" t="n"/>
       <c r="H32" s="11" t="n"/>
       <c r="I32" s="11" t="n"/>
-      <c r="J32" s="11" t="n"/>
+      <c r="J32" s="12">
+        <f>IF(A32="","",COUNTIF(Variants!$A:$A,A32))</f>
+        <v/>
+      </c>
       <c r="K32" s="12">
-        <f>IF(A32="","",COUNTIF(Variants!$A:$A,A32))</f>
+        <f>IF(A32="","",COUNTIFS(Variants!$A:$A,A32,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L32" s="12">
-        <f>IF(A32="","",COUNTIFS(Variants!$A:$A,A32,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M32" s="12">
-        <f>IF(A32="","",IF(K32=0,"ADD VARIANTS",IF(L32&lt;K32,"MISSING "&amp;(K32-L32)&amp;" STORE SKU",IF(E32="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A32="","",IF(J32=0,"ADD VARIANTS",IF(K32&lt;J32,"MISSING "&amp;(J32-K32)&amp;" STORE SKU",IF(D32="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1583,22 +1542,21 @@
       <c r="B33" s="9" t="n"/>
       <c r="C33" s="10" t="n"/>
       <c r="D33" s="9" t="n"/>
-      <c r="E33" s="9" t="n"/>
+      <c r="E33" s="11" t="n"/>
       <c r="F33" s="11" t="n"/>
       <c r="G33" s="11" t="n"/>
       <c r="H33" s="11" t="n"/>
       <c r="I33" s="11" t="n"/>
-      <c r="J33" s="11" t="n"/>
+      <c r="J33" s="12">
+        <f>IF(A33="","",COUNTIF(Variants!$A:$A,A33))</f>
+        <v/>
+      </c>
       <c r="K33" s="12">
-        <f>IF(A33="","",COUNTIF(Variants!$A:$A,A33))</f>
+        <f>IF(A33="","",COUNTIFS(Variants!$A:$A,A33,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L33" s="12">
-        <f>IF(A33="","",COUNTIFS(Variants!$A:$A,A33,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M33" s="12">
-        <f>IF(A33="","",IF(K33=0,"ADD VARIANTS",IF(L33&lt;K33,"MISSING "&amp;(K33-L33)&amp;" STORE SKU",IF(E33="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A33="","",IF(J33=0,"ADD VARIANTS",IF(K33&lt;J33,"MISSING "&amp;(J33-K33)&amp;" STORE SKU",IF(D33="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1607,22 +1565,21 @@
       <c r="B34" s="9" t="n"/>
       <c r="C34" s="10" t="n"/>
       <c r="D34" s="9" t="n"/>
-      <c r="E34" s="9" t="n"/>
+      <c r="E34" s="11" t="n"/>
       <c r="F34" s="11" t="n"/>
       <c r="G34" s="11" t="n"/>
       <c r="H34" s="11" t="n"/>
       <c r="I34" s="11" t="n"/>
-      <c r="J34" s="11" t="n"/>
+      <c r="J34" s="12">
+        <f>IF(A34="","",COUNTIF(Variants!$A:$A,A34))</f>
+        <v/>
+      </c>
       <c r="K34" s="12">
-        <f>IF(A34="","",COUNTIF(Variants!$A:$A,A34))</f>
+        <f>IF(A34="","",COUNTIFS(Variants!$A:$A,A34,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L34" s="12">
-        <f>IF(A34="","",COUNTIFS(Variants!$A:$A,A34,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M34" s="12">
-        <f>IF(A34="","",IF(K34=0,"ADD VARIANTS",IF(L34&lt;K34,"MISSING "&amp;(K34-L34)&amp;" STORE SKU",IF(E34="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A34="","",IF(J34=0,"ADD VARIANTS",IF(K34&lt;J34,"MISSING "&amp;(J34-K34)&amp;" STORE SKU",IF(D34="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1631,22 +1588,21 @@
       <c r="B35" s="9" t="n"/>
       <c r="C35" s="10" t="n"/>
       <c r="D35" s="9" t="n"/>
-      <c r="E35" s="9" t="n"/>
+      <c r="E35" s="11" t="n"/>
       <c r="F35" s="11" t="n"/>
       <c r="G35" s="11" t="n"/>
       <c r="H35" s="11" t="n"/>
       <c r="I35" s="11" t="n"/>
-      <c r="J35" s="11" t="n"/>
+      <c r="J35" s="12">
+        <f>IF(A35="","",COUNTIF(Variants!$A:$A,A35))</f>
+        <v/>
+      </c>
       <c r="K35" s="12">
-        <f>IF(A35="","",COUNTIF(Variants!$A:$A,A35))</f>
+        <f>IF(A35="","",COUNTIFS(Variants!$A:$A,A35,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L35" s="12">
-        <f>IF(A35="","",COUNTIFS(Variants!$A:$A,A35,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M35" s="12">
-        <f>IF(A35="","",IF(K35=0,"ADD VARIANTS",IF(L35&lt;K35,"MISSING "&amp;(K35-L35)&amp;" STORE SKU",IF(E35="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A35="","",IF(J35=0,"ADD VARIANTS",IF(K35&lt;J35,"MISSING "&amp;(J35-K35)&amp;" STORE SKU",IF(D35="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1655,22 +1611,21 @@
       <c r="B36" s="9" t="n"/>
       <c r="C36" s="10" t="n"/>
       <c r="D36" s="9" t="n"/>
-      <c r="E36" s="9" t="n"/>
+      <c r="E36" s="11" t="n"/>
       <c r="F36" s="11" t="n"/>
       <c r="G36" s="11" t="n"/>
       <c r="H36" s="11" t="n"/>
       <c r="I36" s="11" t="n"/>
-      <c r="J36" s="11" t="n"/>
+      <c r="J36" s="12">
+        <f>IF(A36="","",COUNTIF(Variants!$A:$A,A36))</f>
+        <v/>
+      </c>
       <c r="K36" s="12">
-        <f>IF(A36="","",COUNTIF(Variants!$A:$A,A36))</f>
+        <f>IF(A36="","",COUNTIFS(Variants!$A:$A,A36,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L36" s="12">
-        <f>IF(A36="","",COUNTIFS(Variants!$A:$A,A36,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M36" s="12">
-        <f>IF(A36="","",IF(K36=0,"ADD VARIANTS",IF(L36&lt;K36,"MISSING "&amp;(K36-L36)&amp;" STORE SKU",IF(E36="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A36="","",IF(J36=0,"ADD VARIANTS",IF(K36&lt;J36,"MISSING "&amp;(J36-K36)&amp;" STORE SKU",IF(D36="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1679,22 +1634,21 @@
       <c r="B37" s="9" t="n"/>
       <c r="C37" s="10" t="n"/>
       <c r="D37" s="9" t="n"/>
-      <c r="E37" s="9" t="n"/>
+      <c r="E37" s="11" t="n"/>
       <c r="F37" s="11" t="n"/>
       <c r="G37" s="11" t="n"/>
       <c r="H37" s="11" t="n"/>
       <c r="I37" s="11" t="n"/>
-      <c r="J37" s="11" t="n"/>
+      <c r="J37" s="12">
+        <f>IF(A37="","",COUNTIF(Variants!$A:$A,A37))</f>
+        <v/>
+      </c>
       <c r="K37" s="12">
-        <f>IF(A37="","",COUNTIF(Variants!$A:$A,A37))</f>
+        <f>IF(A37="","",COUNTIFS(Variants!$A:$A,A37,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L37" s="12">
-        <f>IF(A37="","",COUNTIFS(Variants!$A:$A,A37,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M37" s="12">
-        <f>IF(A37="","",IF(K37=0,"ADD VARIANTS",IF(L37&lt;K37,"MISSING "&amp;(K37-L37)&amp;" STORE SKU",IF(E37="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A37="","",IF(J37=0,"ADD VARIANTS",IF(K37&lt;J37,"MISSING "&amp;(J37-K37)&amp;" STORE SKU",IF(D37="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1703,22 +1657,21 @@
       <c r="B38" s="9" t="n"/>
       <c r="C38" s="10" t="n"/>
       <c r="D38" s="9" t="n"/>
-      <c r="E38" s="9" t="n"/>
+      <c r="E38" s="11" t="n"/>
       <c r="F38" s="11" t="n"/>
       <c r="G38" s="11" t="n"/>
       <c r="H38" s="11" t="n"/>
       <c r="I38" s="11" t="n"/>
-      <c r="J38" s="11" t="n"/>
+      <c r="J38" s="12">
+        <f>IF(A38="","",COUNTIF(Variants!$A:$A,A38))</f>
+        <v/>
+      </c>
       <c r="K38" s="12">
-        <f>IF(A38="","",COUNTIF(Variants!$A:$A,A38))</f>
+        <f>IF(A38="","",COUNTIFS(Variants!$A:$A,A38,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L38" s="12">
-        <f>IF(A38="","",COUNTIFS(Variants!$A:$A,A38,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M38" s="12">
-        <f>IF(A38="","",IF(K38=0,"ADD VARIANTS",IF(L38&lt;K38,"MISSING "&amp;(K38-L38)&amp;" STORE SKU",IF(E38="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A38="","",IF(J38=0,"ADD VARIANTS",IF(K38&lt;J38,"MISSING "&amp;(J38-K38)&amp;" STORE SKU",IF(D38="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1727,22 +1680,21 @@
       <c r="B39" s="9" t="n"/>
       <c r="C39" s="10" t="n"/>
       <c r="D39" s="9" t="n"/>
-      <c r="E39" s="9" t="n"/>
+      <c r="E39" s="11" t="n"/>
       <c r="F39" s="11" t="n"/>
       <c r="G39" s="11" t="n"/>
       <c r="H39" s="11" t="n"/>
       <c r="I39" s="11" t="n"/>
-      <c r="J39" s="11" t="n"/>
+      <c r="J39" s="12">
+        <f>IF(A39="","",COUNTIF(Variants!$A:$A,A39))</f>
+        <v/>
+      </c>
       <c r="K39" s="12">
-        <f>IF(A39="","",COUNTIF(Variants!$A:$A,A39))</f>
+        <f>IF(A39="","",COUNTIFS(Variants!$A:$A,A39,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L39" s="12">
-        <f>IF(A39="","",COUNTIFS(Variants!$A:$A,A39,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M39" s="12">
-        <f>IF(A39="","",IF(K39=0,"ADD VARIANTS",IF(L39&lt;K39,"MISSING "&amp;(K39-L39)&amp;" STORE SKU",IF(E39="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A39="","",IF(J39=0,"ADD VARIANTS",IF(K39&lt;J39,"MISSING "&amp;(J39-K39)&amp;" STORE SKU",IF(D39="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1751,22 +1703,21 @@
       <c r="B40" s="9" t="n"/>
       <c r="C40" s="10" t="n"/>
       <c r="D40" s="9" t="n"/>
-      <c r="E40" s="9" t="n"/>
+      <c r="E40" s="11" t="n"/>
       <c r="F40" s="11" t="n"/>
       <c r="G40" s="11" t="n"/>
       <c r="H40" s="11" t="n"/>
       <c r="I40" s="11" t="n"/>
-      <c r="J40" s="11" t="n"/>
+      <c r="J40" s="12">
+        <f>IF(A40="","",COUNTIF(Variants!$A:$A,A40))</f>
+        <v/>
+      </c>
       <c r="K40" s="12">
-        <f>IF(A40="","",COUNTIF(Variants!$A:$A,A40))</f>
+        <f>IF(A40="","",COUNTIFS(Variants!$A:$A,A40,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L40" s="12">
-        <f>IF(A40="","",COUNTIFS(Variants!$A:$A,A40,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M40" s="12">
-        <f>IF(A40="","",IF(K40=0,"ADD VARIANTS",IF(L40&lt;K40,"MISSING "&amp;(K40-L40)&amp;" STORE SKU",IF(E40="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A40="","",IF(J40=0,"ADD VARIANTS",IF(K40&lt;J40,"MISSING "&amp;(J40-K40)&amp;" STORE SKU",IF(D40="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1775,22 +1726,21 @@
       <c r="B41" s="9" t="n"/>
       <c r="C41" s="10" t="n"/>
       <c r="D41" s="9" t="n"/>
-      <c r="E41" s="9" t="n"/>
+      <c r="E41" s="11" t="n"/>
       <c r="F41" s="11" t="n"/>
       <c r="G41" s="11" t="n"/>
       <c r="H41" s="11" t="n"/>
       <c r="I41" s="11" t="n"/>
-      <c r="J41" s="11" t="n"/>
+      <c r="J41" s="12">
+        <f>IF(A41="","",COUNTIF(Variants!$A:$A,A41))</f>
+        <v/>
+      </c>
       <c r="K41" s="12">
-        <f>IF(A41="","",COUNTIF(Variants!$A:$A,A41))</f>
+        <f>IF(A41="","",COUNTIFS(Variants!$A:$A,A41,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L41" s="12">
-        <f>IF(A41="","",COUNTIFS(Variants!$A:$A,A41,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M41" s="12">
-        <f>IF(A41="","",IF(K41=0,"ADD VARIANTS",IF(L41&lt;K41,"MISSING "&amp;(K41-L41)&amp;" STORE SKU",IF(E41="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A41="","",IF(J41=0,"ADD VARIANTS",IF(K41&lt;J41,"MISSING "&amp;(J41-K41)&amp;" STORE SKU",IF(D41="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1799,22 +1749,21 @@
       <c r="B42" s="9" t="n"/>
       <c r="C42" s="10" t="n"/>
       <c r="D42" s="9" t="n"/>
-      <c r="E42" s="9" t="n"/>
+      <c r="E42" s="11" t="n"/>
       <c r="F42" s="11" t="n"/>
       <c r="G42" s="11" t="n"/>
       <c r="H42" s="11" t="n"/>
       <c r="I42" s="11" t="n"/>
-      <c r="J42" s="11" t="n"/>
+      <c r="J42" s="12">
+        <f>IF(A42="","",COUNTIF(Variants!$A:$A,A42))</f>
+        <v/>
+      </c>
       <c r="K42" s="12">
-        <f>IF(A42="","",COUNTIF(Variants!$A:$A,A42))</f>
+        <f>IF(A42="","",COUNTIFS(Variants!$A:$A,A42,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L42" s="12">
-        <f>IF(A42="","",COUNTIFS(Variants!$A:$A,A42,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M42" s="12">
-        <f>IF(A42="","",IF(K42=0,"ADD VARIANTS",IF(L42&lt;K42,"MISSING "&amp;(K42-L42)&amp;" STORE SKU",IF(E42="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A42="","",IF(J42=0,"ADD VARIANTS",IF(K42&lt;J42,"MISSING "&amp;(J42-K42)&amp;" STORE SKU",IF(D42="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1823,22 +1772,21 @@
       <c r="B43" s="9" t="n"/>
       <c r="C43" s="10" t="n"/>
       <c r="D43" s="9" t="n"/>
-      <c r="E43" s="9" t="n"/>
+      <c r="E43" s="11" t="n"/>
       <c r="F43" s="11" t="n"/>
       <c r="G43" s="11" t="n"/>
       <c r="H43" s="11" t="n"/>
       <c r="I43" s="11" t="n"/>
-      <c r="J43" s="11" t="n"/>
+      <c r="J43" s="12">
+        <f>IF(A43="","",COUNTIF(Variants!$A:$A,A43))</f>
+        <v/>
+      </c>
       <c r="K43" s="12">
-        <f>IF(A43="","",COUNTIF(Variants!$A:$A,A43))</f>
+        <f>IF(A43="","",COUNTIFS(Variants!$A:$A,A43,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L43" s="12">
-        <f>IF(A43="","",COUNTIFS(Variants!$A:$A,A43,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M43" s="12">
-        <f>IF(A43="","",IF(K43=0,"ADD VARIANTS",IF(L43&lt;K43,"MISSING "&amp;(K43-L43)&amp;" STORE SKU",IF(E43="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A43="","",IF(J43=0,"ADD VARIANTS",IF(K43&lt;J43,"MISSING "&amp;(J43-K43)&amp;" STORE SKU",IF(D43="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1847,22 +1795,21 @@
       <c r="B44" s="9" t="n"/>
       <c r="C44" s="10" t="n"/>
       <c r="D44" s="9" t="n"/>
-      <c r="E44" s="9" t="n"/>
+      <c r="E44" s="11" t="n"/>
       <c r="F44" s="11" t="n"/>
       <c r="G44" s="11" t="n"/>
       <c r="H44" s="11" t="n"/>
       <c r="I44" s="11" t="n"/>
-      <c r="J44" s="11" t="n"/>
+      <c r="J44" s="12">
+        <f>IF(A44="","",COUNTIF(Variants!$A:$A,A44))</f>
+        <v/>
+      </c>
       <c r="K44" s="12">
-        <f>IF(A44="","",COUNTIF(Variants!$A:$A,A44))</f>
+        <f>IF(A44="","",COUNTIFS(Variants!$A:$A,A44,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L44" s="12">
-        <f>IF(A44="","",COUNTIFS(Variants!$A:$A,A44,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M44" s="12">
-        <f>IF(A44="","",IF(K44=0,"ADD VARIANTS",IF(L44&lt;K44,"MISSING "&amp;(K44-L44)&amp;" STORE SKU",IF(E44="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A44="","",IF(J44=0,"ADD VARIANTS",IF(K44&lt;J44,"MISSING "&amp;(J44-K44)&amp;" STORE SKU",IF(D44="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1871,22 +1818,21 @@
       <c r="B45" s="9" t="n"/>
       <c r="C45" s="10" t="n"/>
       <c r="D45" s="9" t="n"/>
-      <c r="E45" s="9" t="n"/>
+      <c r="E45" s="11" t="n"/>
       <c r="F45" s="11" t="n"/>
       <c r="G45" s="11" t="n"/>
       <c r="H45" s="11" t="n"/>
       <c r="I45" s="11" t="n"/>
-      <c r="J45" s="11" t="n"/>
+      <c r="J45" s="12">
+        <f>IF(A45="","",COUNTIF(Variants!$A:$A,A45))</f>
+        <v/>
+      </c>
       <c r="K45" s="12">
-        <f>IF(A45="","",COUNTIF(Variants!$A:$A,A45))</f>
+        <f>IF(A45="","",COUNTIFS(Variants!$A:$A,A45,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L45" s="12">
-        <f>IF(A45="","",COUNTIFS(Variants!$A:$A,A45,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M45" s="12">
-        <f>IF(A45="","",IF(K45=0,"ADD VARIANTS",IF(L45&lt;K45,"MISSING "&amp;(K45-L45)&amp;" STORE SKU",IF(E45="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A45="","",IF(J45=0,"ADD VARIANTS",IF(K45&lt;J45,"MISSING "&amp;(J45-K45)&amp;" STORE SKU",IF(D45="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1895,22 +1841,21 @@
       <c r="B46" s="9" t="n"/>
       <c r="C46" s="10" t="n"/>
       <c r="D46" s="9" t="n"/>
-      <c r="E46" s="9" t="n"/>
+      <c r="E46" s="11" t="n"/>
       <c r="F46" s="11" t="n"/>
       <c r="G46" s="11" t="n"/>
       <c r="H46" s="11" t="n"/>
       <c r="I46" s="11" t="n"/>
-      <c r="J46" s="11" t="n"/>
+      <c r="J46" s="12">
+        <f>IF(A46="","",COUNTIF(Variants!$A:$A,A46))</f>
+        <v/>
+      </c>
       <c r="K46" s="12">
-        <f>IF(A46="","",COUNTIF(Variants!$A:$A,A46))</f>
+        <f>IF(A46="","",COUNTIFS(Variants!$A:$A,A46,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L46" s="12">
-        <f>IF(A46="","",COUNTIFS(Variants!$A:$A,A46,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M46" s="12">
-        <f>IF(A46="","",IF(K46=0,"ADD VARIANTS",IF(L46&lt;K46,"MISSING "&amp;(K46-L46)&amp;" STORE SKU",IF(E46="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A46="","",IF(J46=0,"ADD VARIANTS",IF(K46&lt;J46,"MISSING "&amp;(J46-K46)&amp;" STORE SKU",IF(D46="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1919,22 +1864,21 @@
       <c r="B47" s="9" t="n"/>
       <c r="C47" s="10" t="n"/>
       <c r="D47" s="9" t="n"/>
-      <c r="E47" s="9" t="n"/>
+      <c r="E47" s="11" t="n"/>
       <c r="F47" s="11" t="n"/>
       <c r="G47" s="11" t="n"/>
       <c r="H47" s="11" t="n"/>
       <c r="I47" s="11" t="n"/>
-      <c r="J47" s="11" t="n"/>
+      <c r="J47" s="12">
+        <f>IF(A47="","",COUNTIF(Variants!$A:$A,A47))</f>
+        <v/>
+      </c>
       <c r="K47" s="12">
-        <f>IF(A47="","",COUNTIF(Variants!$A:$A,A47))</f>
+        <f>IF(A47="","",COUNTIFS(Variants!$A:$A,A47,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L47" s="12">
-        <f>IF(A47="","",COUNTIFS(Variants!$A:$A,A47,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M47" s="12">
-        <f>IF(A47="","",IF(K47=0,"ADD VARIANTS",IF(L47&lt;K47,"MISSING "&amp;(K47-L47)&amp;" STORE SKU",IF(E47="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A47="","",IF(J47=0,"ADD VARIANTS",IF(K47&lt;J47,"MISSING "&amp;(J47-K47)&amp;" STORE SKU",IF(D47="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1943,22 +1887,21 @@
       <c r="B48" s="9" t="n"/>
       <c r="C48" s="10" t="n"/>
       <c r="D48" s="9" t="n"/>
-      <c r="E48" s="9" t="n"/>
+      <c r="E48" s="11" t="n"/>
       <c r="F48" s="11" t="n"/>
       <c r="G48" s="11" t="n"/>
       <c r="H48" s="11" t="n"/>
       <c r="I48" s="11" t="n"/>
-      <c r="J48" s="11" t="n"/>
+      <c r="J48" s="12">
+        <f>IF(A48="","",COUNTIF(Variants!$A:$A,A48))</f>
+        <v/>
+      </c>
       <c r="K48" s="12">
-        <f>IF(A48="","",COUNTIF(Variants!$A:$A,A48))</f>
+        <f>IF(A48="","",COUNTIFS(Variants!$A:$A,A48,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L48" s="12">
-        <f>IF(A48="","",COUNTIFS(Variants!$A:$A,A48,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M48" s="12">
-        <f>IF(A48="","",IF(K48=0,"ADD VARIANTS",IF(L48&lt;K48,"MISSING "&amp;(K48-L48)&amp;" STORE SKU",IF(E48="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A48="","",IF(J48=0,"ADD VARIANTS",IF(K48&lt;J48,"MISSING "&amp;(J48-K48)&amp;" STORE SKU",IF(D48="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1967,22 +1910,21 @@
       <c r="B49" s="9" t="n"/>
       <c r="C49" s="10" t="n"/>
       <c r="D49" s="9" t="n"/>
-      <c r="E49" s="9" t="n"/>
+      <c r="E49" s="11" t="n"/>
       <c r="F49" s="11" t="n"/>
       <c r="G49" s="11" t="n"/>
       <c r="H49" s="11" t="n"/>
       <c r="I49" s="11" t="n"/>
-      <c r="J49" s="11" t="n"/>
+      <c r="J49" s="12">
+        <f>IF(A49="","",COUNTIF(Variants!$A:$A,A49))</f>
+        <v/>
+      </c>
       <c r="K49" s="12">
-        <f>IF(A49="","",COUNTIF(Variants!$A:$A,A49))</f>
+        <f>IF(A49="","",COUNTIFS(Variants!$A:$A,A49,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L49" s="12">
-        <f>IF(A49="","",COUNTIFS(Variants!$A:$A,A49,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M49" s="12">
-        <f>IF(A49="","",IF(K49=0,"ADD VARIANTS",IF(L49&lt;K49,"MISSING "&amp;(K49-L49)&amp;" STORE SKU",IF(E49="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A49="","",IF(J49=0,"ADD VARIANTS",IF(K49&lt;J49,"MISSING "&amp;(J49-K49)&amp;" STORE SKU",IF(D49="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -1991,22 +1933,21 @@
       <c r="B50" s="9" t="n"/>
       <c r="C50" s="10" t="n"/>
       <c r="D50" s="9" t="n"/>
-      <c r="E50" s="9" t="n"/>
+      <c r="E50" s="11" t="n"/>
       <c r="F50" s="11" t="n"/>
       <c r="G50" s="11" t="n"/>
       <c r="H50" s="11" t="n"/>
       <c r="I50" s="11" t="n"/>
-      <c r="J50" s="11" t="n"/>
+      <c r="J50" s="12">
+        <f>IF(A50="","",COUNTIF(Variants!$A:$A,A50))</f>
+        <v/>
+      </c>
       <c r="K50" s="12">
-        <f>IF(A50="","",COUNTIF(Variants!$A:$A,A50))</f>
+        <f>IF(A50="","",COUNTIFS(Variants!$A:$A,A50,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L50" s="12">
-        <f>IF(A50="","",COUNTIFS(Variants!$A:$A,A50,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M50" s="12">
-        <f>IF(A50="","",IF(K50=0,"ADD VARIANTS",IF(L50&lt;K50,"MISSING "&amp;(K50-L50)&amp;" STORE SKU",IF(E50="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A50="","",IF(J50=0,"ADD VARIANTS",IF(K50&lt;J50,"MISSING "&amp;(J50-K50)&amp;" STORE SKU",IF(D50="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -2015,22 +1956,21 @@
       <c r="B51" s="9" t="n"/>
       <c r="C51" s="10" t="n"/>
       <c r="D51" s="9" t="n"/>
-      <c r="E51" s="9" t="n"/>
+      <c r="E51" s="11" t="n"/>
       <c r="F51" s="11" t="n"/>
       <c r="G51" s="11" t="n"/>
       <c r="H51" s="11" t="n"/>
       <c r="I51" s="11" t="n"/>
-      <c r="J51" s="11" t="n"/>
+      <c r="J51" s="12">
+        <f>IF(A51="","",COUNTIF(Variants!$A:$A,A51))</f>
+        <v/>
+      </c>
       <c r="K51" s="12">
-        <f>IF(A51="","",COUNTIF(Variants!$A:$A,A51))</f>
+        <f>IF(A51="","",COUNTIFS(Variants!$A:$A,A51,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L51" s="12">
-        <f>IF(A51="","",COUNTIFS(Variants!$A:$A,A51,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M51" s="12">
-        <f>IF(A51="","",IF(K51=0,"ADD VARIANTS",IF(L51&lt;K51,"MISSING "&amp;(K51-L51)&amp;" STORE SKU",IF(E51="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A51="","",IF(J51=0,"ADD VARIANTS",IF(K51&lt;J51,"MISSING "&amp;(J51-K51)&amp;" STORE SKU",IF(D51="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -2039,22 +1979,21 @@
       <c r="B52" s="9" t="n"/>
       <c r="C52" s="10" t="n"/>
       <c r="D52" s="9" t="n"/>
-      <c r="E52" s="9" t="n"/>
+      <c r="E52" s="11" t="n"/>
       <c r="F52" s="11" t="n"/>
       <c r="G52" s="11" t="n"/>
       <c r="H52" s="11" t="n"/>
       <c r="I52" s="11" t="n"/>
-      <c r="J52" s="11" t="n"/>
+      <c r="J52" s="12">
+        <f>IF(A52="","",COUNTIF(Variants!$A:$A,A52))</f>
+        <v/>
+      </c>
       <c r="K52" s="12">
-        <f>IF(A52="","",COUNTIF(Variants!$A:$A,A52))</f>
+        <f>IF(A52="","",COUNTIFS(Variants!$A:$A,A52,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L52" s="12">
-        <f>IF(A52="","",COUNTIFS(Variants!$A:$A,A52,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M52" s="12">
-        <f>IF(A52="","",IF(K52=0,"ADD VARIANTS",IF(L52&lt;K52,"MISSING "&amp;(K52-L52)&amp;" STORE SKU",IF(E52="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A52="","",IF(J52=0,"ADD VARIANTS",IF(K52&lt;J52,"MISSING "&amp;(J52-K52)&amp;" STORE SKU",IF(D52="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -2063,22 +2002,21 @@
       <c r="B53" s="9" t="n"/>
       <c r="C53" s="10" t="n"/>
       <c r="D53" s="9" t="n"/>
-      <c r="E53" s="9" t="n"/>
+      <c r="E53" s="11" t="n"/>
       <c r="F53" s="11" t="n"/>
       <c r="G53" s="11" t="n"/>
       <c r="H53" s="11" t="n"/>
       <c r="I53" s="11" t="n"/>
-      <c r="J53" s="11" t="n"/>
+      <c r="J53" s="12">
+        <f>IF(A53="","",COUNTIF(Variants!$A:$A,A53))</f>
+        <v/>
+      </c>
       <c r="K53" s="12">
-        <f>IF(A53="","",COUNTIF(Variants!$A:$A,A53))</f>
+        <f>IF(A53="","",COUNTIFS(Variants!$A:$A,A53,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L53" s="12">
-        <f>IF(A53="","",COUNTIFS(Variants!$A:$A,A53,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M53" s="12">
-        <f>IF(A53="","",IF(K53=0,"ADD VARIANTS",IF(L53&lt;K53,"MISSING "&amp;(K53-L53)&amp;" STORE SKU",IF(E53="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A53="","",IF(J53=0,"ADD VARIANTS",IF(K53&lt;J53,"MISSING "&amp;(J53-K53)&amp;" STORE SKU",IF(D53="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -2087,22 +2025,21 @@
       <c r="B54" s="9" t="n"/>
       <c r="C54" s="10" t="n"/>
       <c r="D54" s="9" t="n"/>
-      <c r="E54" s="9" t="n"/>
+      <c r="E54" s="11" t="n"/>
       <c r="F54" s="11" t="n"/>
       <c r="G54" s="11" t="n"/>
       <c r="H54" s="11" t="n"/>
       <c r="I54" s="11" t="n"/>
-      <c r="J54" s="11" t="n"/>
+      <c r="J54" s="12">
+        <f>IF(A54="","",COUNTIF(Variants!$A:$A,A54))</f>
+        <v/>
+      </c>
       <c r="K54" s="12">
-        <f>IF(A54="","",COUNTIF(Variants!$A:$A,A54))</f>
+        <f>IF(A54="","",COUNTIFS(Variants!$A:$A,A54,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L54" s="12">
-        <f>IF(A54="","",COUNTIFS(Variants!$A:$A,A54,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M54" s="12">
-        <f>IF(A54="","",IF(K54=0,"ADD VARIANTS",IF(L54&lt;K54,"MISSING "&amp;(K54-L54)&amp;" STORE SKU",IF(E54="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A54="","",IF(J54=0,"ADD VARIANTS",IF(K54&lt;J54,"MISSING "&amp;(J54-K54)&amp;" STORE SKU",IF(D54="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -2111,22 +2048,21 @@
       <c r="B55" s="9" t="n"/>
       <c r="C55" s="10" t="n"/>
       <c r="D55" s="9" t="n"/>
-      <c r="E55" s="9" t="n"/>
+      <c r="E55" s="11" t="n"/>
       <c r="F55" s="11" t="n"/>
       <c r="G55" s="11" t="n"/>
       <c r="H55" s="11" t="n"/>
       <c r="I55" s="11" t="n"/>
-      <c r="J55" s="11" t="n"/>
+      <c r="J55" s="12">
+        <f>IF(A55="","",COUNTIF(Variants!$A:$A,A55))</f>
+        <v/>
+      </c>
       <c r="K55" s="12">
-        <f>IF(A55="","",COUNTIF(Variants!$A:$A,A55))</f>
+        <f>IF(A55="","",COUNTIFS(Variants!$A:$A,A55,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L55" s="12">
-        <f>IF(A55="","",COUNTIFS(Variants!$A:$A,A55,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M55" s="12">
-        <f>IF(A55="","",IF(K55=0,"ADD VARIANTS",IF(L55&lt;K55,"MISSING "&amp;(K55-L55)&amp;" STORE SKU",IF(E55="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A55="","",IF(J55=0,"ADD VARIANTS",IF(K55&lt;J55,"MISSING "&amp;(J55-K55)&amp;" STORE SKU",IF(D55="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -2135,22 +2071,21 @@
       <c r="B56" s="9" t="n"/>
       <c r="C56" s="10" t="n"/>
       <c r="D56" s="9" t="n"/>
-      <c r="E56" s="9" t="n"/>
+      <c r="E56" s="11" t="n"/>
       <c r="F56" s="11" t="n"/>
       <c r="G56" s="11" t="n"/>
       <c r="H56" s="11" t="n"/>
       <c r="I56" s="11" t="n"/>
-      <c r="J56" s="11" t="n"/>
+      <c r="J56" s="12">
+        <f>IF(A56="","",COUNTIF(Variants!$A:$A,A56))</f>
+        <v/>
+      </c>
       <c r="K56" s="12">
-        <f>IF(A56="","",COUNTIF(Variants!$A:$A,A56))</f>
+        <f>IF(A56="","",COUNTIFS(Variants!$A:$A,A56,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L56" s="12">
-        <f>IF(A56="","",COUNTIFS(Variants!$A:$A,A56,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M56" s="12">
-        <f>IF(A56="","",IF(K56=0,"ADD VARIANTS",IF(L56&lt;K56,"MISSING "&amp;(K56-L56)&amp;" STORE SKU",IF(E56="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A56="","",IF(J56=0,"ADD VARIANTS",IF(K56&lt;J56,"MISSING "&amp;(J56-K56)&amp;" STORE SKU",IF(D56="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -2159,22 +2094,21 @@
       <c r="B57" s="9" t="n"/>
       <c r="C57" s="10" t="n"/>
       <c r="D57" s="9" t="n"/>
-      <c r="E57" s="9" t="n"/>
+      <c r="E57" s="11" t="n"/>
       <c r="F57" s="11" t="n"/>
       <c r="G57" s="11" t="n"/>
       <c r="H57" s="11" t="n"/>
       <c r="I57" s="11" t="n"/>
-      <c r="J57" s="11" t="n"/>
+      <c r="J57" s="12">
+        <f>IF(A57="","",COUNTIF(Variants!$A:$A,A57))</f>
+        <v/>
+      </c>
       <c r="K57" s="12">
-        <f>IF(A57="","",COUNTIF(Variants!$A:$A,A57))</f>
+        <f>IF(A57="","",COUNTIFS(Variants!$A:$A,A57,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L57" s="12">
-        <f>IF(A57="","",COUNTIFS(Variants!$A:$A,A57,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M57" s="12">
-        <f>IF(A57="","",IF(K57=0,"ADD VARIANTS",IF(L57&lt;K57,"MISSING "&amp;(K57-L57)&amp;" STORE SKU",IF(E57="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A57="","",IF(J57=0,"ADD VARIANTS",IF(K57&lt;J57,"MISSING "&amp;(J57-K57)&amp;" STORE SKU",IF(D57="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -2183,22 +2117,21 @@
       <c r="B58" s="9" t="n"/>
       <c r="C58" s="10" t="n"/>
       <c r="D58" s="9" t="n"/>
-      <c r="E58" s="9" t="n"/>
+      <c r="E58" s="11" t="n"/>
       <c r="F58" s="11" t="n"/>
       <c r="G58" s="11" t="n"/>
       <c r="H58" s="11" t="n"/>
       <c r="I58" s="11" t="n"/>
-      <c r="J58" s="11" t="n"/>
+      <c r="J58" s="12">
+        <f>IF(A58="","",COUNTIF(Variants!$A:$A,A58))</f>
+        <v/>
+      </c>
       <c r="K58" s="12">
-        <f>IF(A58="","",COUNTIF(Variants!$A:$A,A58))</f>
+        <f>IF(A58="","",COUNTIFS(Variants!$A:$A,A58,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L58" s="12">
-        <f>IF(A58="","",COUNTIFS(Variants!$A:$A,A58,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M58" s="12">
-        <f>IF(A58="","",IF(K58=0,"ADD VARIANTS",IF(L58&lt;K58,"MISSING "&amp;(K58-L58)&amp;" STORE SKU",IF(E58="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A58="","",IF(J58=0,"ADD VARIANTS",IF(K58&lt;J58,"MISSING "&amp;(J58-K58)&amp;" STORE SKU",IF(D58="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -2207,22 +2140,21 @@
       <c r="B59" s="9" t="n"/>
       <c r="C59" s="10" t="n"/>
       <c r="D59" s="9" t="n"/>
-      <c r="E59" s="9" t="n"/>
+      <c r="E59" s="11" t="n"/>
       <c r="F59" s="11" t="n"/>
       <c r="G59" s="11" t="n"/>
       <c r="H59" s="11" t="n"/>
       <c r="I59" s="11" t="n"/>
-      <c r="J59" s="11" t="n"/>
+      <c r="J59" s="12">
+        <f>IF(A59="","",COUNTIF(Variants!$A:$A,A59))</f>
+        <v/>
+      </c>
       <c r="K59" s="12">
-        <f>IF(A59="","",COUNTIF(Variants!$A:$A,A59))</f>
+        <f>IF(A59="","",COUNTIFS(Variants!$A:$A,A59,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L59" s="12">
-        <f>IF(A59="","",COUNTIFS(Variants!$A:$A,A59,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M59" s="12">
-        <f>IF(A59="","",IF(K59=0,"ADD VARIANTS",IF(L59&lt;K59,"MISSING "&amp;(K59-L59)&amp;" STORE SKU",IF(E59="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A59="","",IF(J59=0,"ADD VARIANTS",IF(K59&lt;J59,"MISSING "&amp;(J59-K59)&amp;" STORE SKU",IF(D59="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
@@ -2231,30 +2163,26 @@
       <c r="B60" s="9" t="n"/>
       <c r="C60" s="10" t="n"/>
       <c r="D60" s="9" t="n"/>
-      <c r="E60" s="9" t="n"/>
+      <c r="E60" s="11" t="n"/>
       <c r="F60" s="11" t="n"/>
       <c r="G60" s="11" t="n"/>
       <c r="H60" s="11" t="n"/>
       <c r="I60" s="11" t="n"/>
-      <c r="J60" s="11" t="n"/>
+      <c r="J60" s="12">
+        <f>IF(A60="","",COUNTIF(Variants!$A:$A,A60))</f>
+        <v/>
+      </c>
       <c r="K60" s="12">
-        <f>IF(A60="","",COUNTIF(Variants!$A:$A,A60))</f>
+        <f>IF(A60="","",COUNTIFS(Variants!$A:$A,A60,Variants!$D:$D,"&lt;&gt;"))</f>
         <v/>
       </c>
       <c r="L60" s="12">
-        <f>IF(A60="","",COUNTIFS(Variants!$A:$A,A60,Variants!$D:$D,"&lt;&gt;"))</f>
-        <v/>
-      </c>
-      <c r="M60" s="12">
-        <f>IF(A60="","",IF(K60=0,"ADD VARIANTS",IF(L60&lt;K60,"MISSING "&amp;(K60-L60)&amp;" STORE SKU",IF(E60="","ADD COVER IMAGE","READY"))))</f>
+        <f>IF(A60="","",IF(J60=0,"ADD VARIANTS",IF(K60&lt;J60,"MISSING "&amp;(J60-K60)&amp;" STORE SKU",IF(D60="","ADD COVER IMAGE","READY"))))</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation sqref="D2:D60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Lists!$B$2:$B$3</formula1>
-    </dataValidation>
+  <dataValidations count="1">
     <dataValidation sqref="C2:C60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Price" error="Enter the selling price in rupees, e.g. 599." type="decimal" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
@@ -2363,11 +2291,7 @@
           <t>v-9Rqh0iKDaVZW18UNNhEhubTepA3d8nuc</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>https://qikink-assets.s3.ap-south-1.amazonaws.com/clients/621544/clientProducts/32422268/images/Front_1_c_1.jpg</t>
-        </is>
-      </c>
+      <c r="E2" s="11" t="n"/>
       <c r="F2" s="13" t="n"/>
       <c r="G2" s="11" t="inlineStr">
         <is>
@@ -2411,11 +2335,7 @@
           <t>v-9Rqh0iKDaVZW18UNNhEhubTepA3d8nud</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>https://qikink-assets.s3.ap-south-1.amazonaws.com/clients/621544/clientProducts/32422268/images/Front_1_c_1.jpg</t>
-        </is>
-      </c>
+      <c r="E3" s="11" t="n"/>
       <c r="F3" s="13" t="n"/>
       <c r="G3" s="11" t="inlineStr">
         <is>
@@ -2459,11 +2379,7 @@
           <t>v-9Rqh0iKDaVZW18UNNhEhubTepA3d8nue</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>https://qikink-assets.s3.ap-south-1.amazonaws.com/clients/621544/clientProducts/32422268/images/Front_1_c_1.jpg</t>
-        </is>
-      </c>
+      <c r="E4" s="11" t="n"/>
       <c r="F4" s="13" t="n"/>
       <c r="G4" s="11" t="inlineStr">
         <is>
@@ -2507,11 +2423,7 @@
           <t>v-9Rqh0iKDaVZW18UNNhEhubTepA3d8nuf</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>https://qikink-assets.s3.ap-south-1.amazonaws.com/clients/621544/clientProducts/32422268/images/Front_1_c_1.jpg</t>
-        </is>
-      </c>
+      <c r="E5" s="11" t="n"/>
       <c r="F5" s="13" t="n"/>
       <c r="G5" s="11" t="inlineStr">
         <is>
@@ -15819,12 +15731,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -15835,11 +15746,6 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>Statuses</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
           <t>Common colours (you can type others)</t>
         </is>
       </c>
@@ -15852,11 +15758,6 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
           <t>White</t>
         </is>
       </c>
@@ -15869,11 +15770,6 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
           <t>Black</t>
         </is>
       </c>
@@ -15884,7 +15780,7 @@
           <t>M</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Navy Blue</t>
         </is>
@@ -15896,7 +15792,7 @@
           <t>L</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Grey Melange</t>
         </is>
@@ -15908,7 +15804,7 @@
           <t>XL</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Maroon</t>
         </is>
@@ -15920,7 +15816,7 @@
           <t>XXL</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Bottle Green</t>
         </is>
@@ -15932,7 +15828,7 @@
           <t>3XL</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Royal Blue</t>
         </is>
@@ -15944,7 +15840,7 @@
           <t>4XL</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -15956,7 +15852,7 @@
           <t>5XL</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Yellow</t>
         </is>
@@ -15968,42 +15864,42 @@
           <t>Free Size</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Olive Green</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="C12" s="3" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Beige</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="C13" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Lavender</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="C14" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Baby Pink</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="C15" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Sky Blue</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="C16" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Charcoal Melange</t>
         </is>

</xml_diff>

<commit_message>
Restore the White colour images in the product sheet template.
Dropping the Status column shifted the cover image column, so the example
White rows lost their colour image.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/SunoBro-Product-Sheet.xlsx
+++ b/public/SunoBro-Product-Sheet.xlsx
@@ -2291,7 +2291,11 @@
           <t>v-9Rqh0iKDaVZW18UNNhEhubTepA3d8nuc</t>
         </is>
       </c>
-      <c r="E2" s="11" t="n"/>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>https://qikink-assets.s3.ap-south-1.amazonaws.com/clients/621544/clientProducts/32422268/images/Front_1_c_1.jpg</t>
+        </is>
+      </c>
       <c r="F2" s="13" t="n"/>
       <c r="G2" s="11" t="inlineStr">
         <is>
@@ -2335,7 +2339,11 @@
           <t>v-9Rqh0iKDaVZW18UNNhEhubTepA3d8nud</t>
         </is>
       </c>
-      <c r="E3" s="11" t="n"/>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>https://qikink-assets.s3.ap-south-1.amazonaws.com/clients/621544/clientProducts/32422268/images/Front_1_c_1.jpg</t>
+        </is>
+      </c>
       <c r="F3" s="13" t="n"/>
       <c r="G3" s="11" t="inlineStr">
         <is>
@@ -2379,7 +2387,11 @@
           <t>v-9Rqh0iKDaVZW18UNNhEhubTepA3d8nue</t>
         </is>
       </c>
-      <c r="E4" s="11" t="n"/>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>https://qikink-assets.s3.ap-south-1.amazonaws.com/clients/621544/clientProducts/32422268/images/Front_1_c_1.jpg</t>
+        </is>
+      </c>
       <c r="F4" s="13" t="n"/>
       <c r="G4" s="11" t="inlineStr">
         <is>
@@ -2423,7 +2435,11 @@
           <t>v-9Rqh0iKDaVZW18UNNhEhubTepA3d8nuf</t>
         </is>
       </c>
-      <c r="E5" s="11" t="n"/>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>https://qikink-assets.s3.ap-south-1.amazonaws.com/clients/621544/clientProducts/32422268/images/Front_1_c_1.jpg</t>
+        </is>
+      </c>
       <c r="F5" s="13" t="n"/>
       <c r="G5" s="11" t="inlineStr">
         <is>

</xml_diff>